<commit_message>
feat(visualization): enhance plot layout and add GitHub Pages support
Visualization improvements:
- Move subplot titles inside graphs (top center annotation)
- Remove y-axis labels from right column to prevent overlap
- Move colorbar to horizontal position above first graph
- Simplify legend: only "Měření" and "Outlier" shown
- Move RMSE legend inside graph (top-right corner)
- Adjust spacing: horizontal_spacing=0.12, vertical_spacing=0.06

GitHub Pages:
- Add docs/ folder with interactive comparison plot
- Copy comparison_results_plot.html as docs/index.html

Configuration:
- Update .gitignore: exclude pandoc-3.8.3/ and report/
</commit_message>
<xml_diff>
--- a/data_analysis/output/comparison_input.xlsx
+++ b/data_analysis/output/comparison_input.xlsx
@@ -577,7 +577,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -628,7 +628,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -716,7 +716,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -767,7 +767,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -859,7 +859,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -910,7 +910,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H19" t="n">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -1717,7 +1717,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H28" t="n">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H31" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H34" t="n">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H36" t="n">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H37" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H39" t="n">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H40" t="n">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H42" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H43" t="n">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H46" t="n">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H48" t="n">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H49" t="n">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H51" t="n">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H52" t="n">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H54" t="n">
@@ -3055,7 +3055,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H55" t="n">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H57" t="n">
@@ -3198,7 +3198,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H58" t="n">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H60" t="n">
@@ -3341,7 +3341,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H61" t="n">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H63" t="n">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H64" t="n">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H66" t="n">
@@ -3627,7 +3627,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H67" t="n">
@@ -3719,7 +3719,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H69" t="n">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H70" t="n">
@@ -3862,7 +3862,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H72" t="n">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H73" t="n">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H75" t="n">
@@ -4056,7 +4056,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H76" t="n">
@@ -4148,7 +4148,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H78" t="n">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H79" t="n">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H81" t="n">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H82" t="n">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H84" t="n">
@@ -4485,7 +4485,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H85" t="n">
@@ -4577,7 +4577,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H87" t="n">
@@ -4628,7 +4628,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H88" t="n">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H90" t="n">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -4863,7 +4863,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H93" t="n">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H94" t="n">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H96" t="n">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H97" t="n">
@@ -5149,7 +5149,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H99" t="n">
@@ -5200,7 +5200,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H100" t="n">
@@ -5292,7 +5292,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H102" t="n">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H103" t="n">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H105" t="n">
@@ -5486,7 +5486,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H106" t="n">
@@ -5578,7 +5578,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H108" t="n">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H109" t="n">
@@ -5721,7 +5721,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H111" t="n">
@@ -5772,7 +5772,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H112" t="n">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H114" t="n">
@@ -5915,7 +5915,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H115" t="n">
@@ -6007,7 +6007,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H117" t="n">
@@ -6058,7 +6058,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H118" t="n">
@@ -6150,7 +6150,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H120" t="n">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H121" t="n">
@@ -6293,7 +6293,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H123" t="n">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H124" t="n">
@@ -6436,7 +6436,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H126" t="n">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H127" t="n">
@@ -6579,7 +6579,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H129" t="n">
@@ -6630,7 +6630,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H130" t="n">
@@ -6722,7 +6722,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H132" t="n">
@@ -6773,7 +6773,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H133" t="n">
@@ -6865,7 +6865,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H135" t="n">
@@ -6916,7 +6916,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H136" t="n">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H138" t="n">
@@ -7059,7 +7059,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H139" t="n">
@@ -7151,7 +7151,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H141" t="n">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H142" t="n">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H144" t="n">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H145" t="n">
@@ -7437,7 +7437,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H147" t="n">
@@ -7488,7 +7488,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H148" t="n">
@@ -7580,7 +7580,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H150" t="n">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H151" t="n">
@@ -7723,7 +7723,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H153" t="n">
@@ -7774,7 +7774,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H154" t="n">
@@ -7866,7 +7866,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H156" t="n">
@@ -7917,7 +7917,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H157" t="n">
@@ -8009,7 +8009,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H159" t="n">
@@ -8060,7 +8060,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H160" t="n">
@@ -8152,7 +8152,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H162" t="n">
@@ -8203,7 +8203,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H163" t="n">
@@ -8295,7 +8295,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H165" t="n">
@@ -8346,7 +8346,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H166" t="n">
@@ -8438,7 +8438,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H168" t="n">
@@ -8489,7 +8489,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H169" t="n">
@@ -8581,7 +8581,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H171" t="n">
@@ -8632,7 +8632,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H172" t="n">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H174" t="n">
@@ -8775,7 +8775,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H175" t="n">
@@ -8867,7 +8867,7 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H177" t="n">
@@ -8918,7 +8918,7 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H178" t="n">
@@ -9010,7 +9010,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H180" t="n">
@@ -9061,7 +9061,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H181" t="n">
@@ -9153,7 +9153,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H183" t="n">
@@ -9204,7 +9204,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H184" t="n">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H186" t="n">
@@ -9347,7 +9347,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H187" t="n">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H189" t="n">
@@ -9490,7 +9490,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H190" t="n">
@@ -9582,7 +9582,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H192" t="n">
@@ -9633,7 +9633,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H193" t="n">
@@ -9725,7 +9725,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H195" t="n">
@@ -9776,7 +9776,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H196" t="n">
@@ -9868,7 +9868,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H198" t="n">
@@ -9919,7 +9919,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H199" t="n">
@@ -10011,7 +10011,7 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H201" t="n">
@@ -10062,7 +10062,7 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H202" t="n">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H204" t="n">
@@ -10205,7 +10205,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H205" t="n">
@@ -10297,7 +10297,7 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H207" t="n">
@@ -10348,7 +10348,7 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H208" t="n">
@@ -10440,7 +10440,7 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H210" t="n">
@@ -10491,7 +10491,7 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H211" t="n">
@@ -10583,7 +10583,7 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H213" t="n">
@@ -10634,7 +10634,7 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H214" t="n">
@@ -10726,7 +10726,7 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H216" t="n">
@@ -10777,7 +10777,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H217" t="n">
@@ -10869,7 +10869,7 @@
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H219" t="n">
@@ -10920,7 +10920,7 @@
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H220" t="n">
@@ -11012,7 +11012,7 @@
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H222" t="n">
@@ -11063,7 +11063,7 @@
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>2026-01-07</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="H223" t="n">

</xml_diff>